<commit_message>
Add and update files mmei 06052026
</commit_message>
<xml_diff>
--- a/data_operasi_reaktor2/Data Reaktor Kartini_11-02-26.xlsx
+++ b/data_operasi_reaktor2/Data Reaktor Kartini_11-02-26.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Kuliah S3 TPU\Kartini Reactor\data_operasi_reaktor2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3962D2C-F96E-47E3-8E4B-F5CE37751832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86C08144-336C-4CDC-A0D9-501335C0028C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{B92E438E-36C7-4333-ACE8-EBB87BB02489}"/>
   </bookViews>
@@ -51,6 +51,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="#,##0.000"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -80,11 +83,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -419,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEC4857B-21DD-4ECC-AD26-213FEE62CD70}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -584,6 +588,9 @@
       <c r="D12">
         <v>68</v>
       </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B14" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>